<commit_message>
Configure admin email allowlist
</commit_message>
<xml_diff>
--- a/docs/AWS_DEPLOYMENT_MANAGEMENT_SAFE.xlsx
+++ b/docs/AWS_DEPLOYMENT_MANAGEMENT_SAFE.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rd999c665afbb41b9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resources" sheetId="2" r:id="R7d519017eb9a4fbb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Env_and_Secrets" sheetId="3" r:id="R433e961c6a1b47e3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Publish_Flow" sheetId="4" r:id="R14519227fe914867"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Console_URLs" sheetId="5" r:id="R4b3f429e53ea446a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rdd2f202a225f44e0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resources" sheetId="2" r:id="Rdbe6e1ba8b6947bb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Env_and_Secrets" sheetId="3" r:id="R101402fb550144bc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Publish_Flow" sheetId="4" r:id="R95e1145ce2024c2f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Console_URLs" sheetId="5" r:id="Rbaa3c6e57cae432d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1194,112 +1194,110 @@
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="4" t="str">
-        <x:v>Database password</x:v>
+        <x:v>Admin email allowlist</x:v>
       </x:c>
       <x:c r="B10" s="4" t="str">
-        <x:v>Secret</x:v>
+        <x:v>Plain env</x:v>
       </x:c>
       <x:c r="C10" s="4" t="str">
-        <x:v>PGPASSWORD</x:v>
+        <x:v>ADMIN_EMAILS</x:v>
       </x:c>
       <x:c r="D10" s="4" t="str">
-        <x:v>NOT RECORDED</x:v>
-      </x:c>
-      <x:c r="E10" s="4" t="str">
-        <x:v>Test_DB</x:v>
-      </x:c>
-      <x:c r="F10" s="4" t="str">
-        <x:v>password</x:v>
-      </x:c>
+        <x:v>haohan6037@gmail.com,kaiyu.yang@youngproperty.co.nz</x:v>
+      </x:c>
+      <x:c r="E10" s="4" t="str"/>
+      <x:c r="F10" s="4" t="str"/>
       <x:c r="G10" s="4" t="str">
-        <x:v>ECS secret injection</x:v>
+        <x:v>ECS task definition</x:v>
       </x:c>
       <x:c r="H10" s="4" t="str">
-        <x:v>Safe: records secret reference only</x:v>
+        <x:v>Safe</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="4" t="str">
-        <x:v>Geoapify API key</x:v>
+        <x:v>Provider email allowlist</x:v>
       </x:c>
       <x:c r="B11" s="4" t="str">
-        <x:v>Secret</x:v>
+        <x:v>Plain env</x:v>
       </x:c>
       <x:c r="C11" s="4" t="str">
-        <x:v>GEOAPIFY_API_KEY</x:v>
-      </x:c>
-      <x:c r="D11" s="4" t="str">
-        <x:v>NOT RECORDED</x:v>
-      </x:c>
-      <x:c r="E11" s="4" t="str">
-        <x:v>Geoapify</x:v>
-      </x:c>
-      <x:c r="F11" s="4" t="str">
-        <x:v>GEOAPIFY_API_KEY</x:v>
-      </x:c>
+        <x:v>PROVIDER_EMAILS</x:v>
+      </x:c>
+      <x:c r="D11" s="4" t="str"/>
+      <x:c r="E11" s="4" t="str"/>
+      <x:c r="F11" s="4" t="str"/>
       <x:c r="G11" s="4" t="str">
-        <x:v>ECS secret injection</x:v>
+        <x:v>ECS task definition</x:v>
       </x:c>
       <x:c r="H11" s="4" t="str">
-        <x:v>Safe: records secret reference only</x:v>
+        <x:v>Safe</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="4" t="str">
-        <x:v>AWS deploy role</x:v>
+        <x:v>Database password</x:v>
       </x:c>
       <x:c r="B12" s="4" t="str">
-        <x:v>GitHub variable</x:v>
+        <x:v>Secret</x:v>
       </x:c>
       <x:c r="C12" s="4" t="str">
-        <x:v>AWS_DEPLOY_ROLE_ARN</x:v>
+        <x:v>PGPASSWORD</x:v>
       </x:c>
       <x:c r="D12" s="4" t="str">
-        <x:v>Role ARN only</x:v>
-      </x:c>
-      <x:c r="E12" s="4" t="str"/>
-      <x:c r="F12" s="4" t="str"/>
+        <x:v>NOT RECORDED</x:v>
+      </x:c>
+      <x:c r="E12" s="4" t="str">
+        <x:v>Test_DB</x:v>
+      </x:c>
+      <x:c r="F12" s="4" t="str">
+        <x:v>password</x:v>
+      </x:c>
       <x:c r="G12" s="4" t="str">
-        <x:v>GitHub Actions test environment</x:v>
+        <x:v>ECS secret injection</x:v>
       </x:c>
       <x:c r="H12" s="4" t="str">
-        <x:v>Safe</x:v>
+        <x:v>Safe: records secret reference only</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="4" t="str">
-        <x:v>ECR repository</x:v>
+        <x:v>Geoapify API key</x:v>
       </x:c>
       <x:c r="B13" s="4" t="str">
-        <x:v>GitHub variable</x:v>
+        <x:v>Secret</x:v>
       </x:c>
       <x:c r="C13" s="4" t="str">
-        <x:v>ECR_REPOSITORY</x:v>
+        <x:v>GEOAPIFY_API_KEY</x:v>
       </x:c>
       <x:c r="D13" s="4" t="str">
-        <x:v>gardenos-test-app</x:v>
-      </x:c>
-      <x:c r="E13" s="4" t="str"/>
-      <x:c r="F13" s="4" t="str"/>
+        <x:v>NOT RECORDED</x:v>
+      </x:c>
+      <x:c r="E13" s="4" t="str">
+        <x:v>Geoapify</x:v>
+      </x:c>
+      <x:c r="F13" s="4" t="str">
+        <x:v>GEOAPIFY_API_KEY</x:v>
+      </x:c>
       <x:c r="G13" s="4" t="str">
-        <x:v>GitHub Actions test environment</x:v>
+        <x:v>ECS secret injection</x:v>
       </x:c>
       <x:c r="H13" s="4" t="str">
-        <x:v>Safe</x:v>
+        <x:v>Safe: records secret reference only</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="4" t="str">
-        <x:v>ECS cluster</x:v>
+        <x:v>AWS deploy role</x:v>
       </x:c>
       <x:c r="B14" s="4" t="str">
         <x:v>GitHub variable</x:v>
       </x:c>
       <x:c r="C14" s="4" t="str">
-        <x:v>ECS_CLUSTER</x:v>
+        <x:v>AWS_DEPLOY_ROLE_ARN</x:v>
       </x:c>
       <x:c r="D14" s="4" t="str">
-        <x:v>gardenos-test</x:v>
+        <x:v>Role ARN only</x:v>
       </x:c>
       <x:c r="E14" s="4" t="str"/>
       <x:c r="F14" s="4" t="str"/>
@@ -1312,16 +1310,16 @@
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="4" t="str">
-        <x:v>ECS service</x:v>
+        <x:v>ECR repository</x:v>
       </x:c>
       <x:c r="B15" s="4" t="str">
         <x:v>GitHub variable</x:v>
       </x:c>
       <x:c r="C15" s="4" t="str">
-        <x:v>ECS_SERVICE</x:v>
+        <x:v>ECR_REPOSITORY</x:v>
       </x:c>
       <x:c r="D15" s="4" t="str">
-        <x:v>gardenos-test</x:v>
+        <x:v>gardenos-test-app</x:v>
       </x:c>
       <x:c r="E15" s="4" t="str"/>
       <x:c r="F15" s="4" t="str"/>
@@ -1334,13 +1332,13 @@
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="4" t="str">
-        <x:v>Task definition family</x:v>
+        <x:v>ECS cluster</x:v>
       </x:c>
       <x:c r="B16" s="4" t="str">
         <x:v>GitHub variable</x:v>
       </x:c>
       <x:c r="C16" s="4" t="str">
-        <x:v>ECS_TASK_DEFINITION_FAMILY</x:v>
+        <x:v>ECS_CLUSTER</x:v>
       </x:c>
       <x:c r="D16" s="4" t="str">
         <x:v>gardenos-test</x:v>
@@ -1351,6 +1349,50 @@
         <x:v>GitHub Actions test environment</x:v>
       </x:c>
       <x:c r="H16" s="4" t="str">
+        <x:v>Safe</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="4" t="str">
+        <x:v>ECS service</x:v>
+      </x:c>
+      <x:c r="B17" s="4" t="str">
+        <x:v>GitHub variable</x:v>
+      </x:c>
+      <x:c r="C17" s="4" t="str">
+        <x:v>ECS_SERVICE</x:v>
+      </x:c>
+      <x:c r="D17" s="4" t="str">
+        <x:v>gardenos-test</x:v>
+      </x:c>
+      <x:c r="E17" s="4" t="str"/>
+      <x:c r="F17" s="4" t="str"/>
+      <x:c r="G17" s="4" t="str">
+        <x:v>GitHub Actions test environment</x:v>
+      </x:c>
+      <x:c r="H17" s="4" t="str">
+        <x:v>Safe</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="4" t="str">
+        <x:v>Task definition family</x:v>
+      </x:c>
+      <x:c r="B18" s="4" t="str">
+        <x:v>GitHub variable</x:v>
+      </x:c>
+      <x:c r="C18" s="4" t="str">
+        <x:v>ECS_TASK_DEFINITION_FAMILY</x:v>
+      </x:c>
+      <x:c r="D18" s="4" t="str">
+        <x:v>gardenos-test</x:v>
+      </x:c>
+      <x:c r="E18" s="4" t="str"/>
+      <x:c r="F18" s="4" t="str"/>
+      <x:c r="G18" s="4" t="str">
+        <x:v>GitHub Actions test environment</x:v>
+      </x:c>
+      <x:c r="H18" s="4" t="str">
         <x:v>Safe</x:v>
       </x:c>
     </x:row>

</xml_diff>